<commit_message>
incorporating Pemba feedback to death report - ZN-232 (#96)
* incorporating Pemba feedback to death report - ZN-232
* fix relevancy condition to only include female clients >12
* swapped initial question to probe for reason of death
</commit_message>
<xml_diff>
--- a/forms/app/death_report.xlsx
+++ b/forms/app/death_report.xlsx
@@ -13,18 +13,33 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="200">
+  <si>
+    <t>list_name</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>label::en</t>
+  </si>
+  <si>
+    <t>label::sw</t>
+  </si>
+  <si>
+    <t>yes_no</t>
+  </si>
   <si>
     <t>type</t>
   </si>
   <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>label::en</t>
-  </si>
-  <si>
-    <t>label::sw</t>
+    <t>form_title</t>
+  </si>
+  <si>
+    <t>form_id</t>
+  </si>
+  <si>
+    <t>version</t>
   </si>
   <si>
     <t>required</t>
@@ -45,66 +60,63 @@
     <t>constraint_message::en</t>
   </si>
   <si>
-    <t>form_title</t>
-  </si>
-  <si>
-    <t>list_name</t>
-  </si>
-  <si>
-    <t>form_id</t>
-  </si>
-  <si>
-    <t>version</t>
+    <t>constraint_message::sw</t>
+  </si>
+  <si>
+    <t>calculation</t>
+  </si>
+  <si>
+    <t>choice_filter</t>
+  </si>
+  <si>
+    <t>hint::en</t>
+  </si>
+  <si>
+    <t>hint::sw</t>
+  </si>
+  <si>
+    <t>default</t>
   </si>
   <si>
     <t>style</t>
   </si>
   <si>
+    <t>yes</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
     <t>instance_name</t>
   </si>
   <si>
-    <t>yes_no</t>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Ndiyo</t>
   </si>
   <si>
     <t>Death Report</t>
   </si>
   <si>
-    <t>constraint_message::sw</t>
-  </si>
-  <si>
-    <t>calculation</t>
-  </si>
-  <si>
-    <t>choice_filter</t>
-  </si>
-  <si>
-    <t>hint::en</t>
-  </si>
-  <si>
-    <t>hint::sw</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
     <t>death_report</t>
   </si>
   <si>
-    <t>default</t>
-  </si>
-  <si>
-    <t>Yes</t>
+    <t>no</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Hapana</t>
+  </si>
+  <si>
+    <t>yes_no_dontknow</t>
   </si>
   <si>
     <t>repeat_count</t>
   </si>
   <si>
-    <t>Ndiyo</t>
-  </si>
-  <si>
     <t>begin group</t>
   </si>
   <si>
@@ -114,21 +126,108 @@
     <t>NO_LABEL</t>
   </si>
   <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Hapana</t>
-  </si>
-  <si>
-    <t>when_death</t>
+    <t>dont_know</t>
+  </si>
+  <si>
+    <t>I don't know</t>
+  </si>
+  <si>
+    <t>Sijui</t>
+  </si>
+  <si>
+    <t>reason_death</t>
+  </si>
+  <si>
+    <t>pregnancy_delivery</t>
+  </si>
+  <si>
+    <t>Death related to pregnancy or recent delivery</t>
+  </si>
+  <si>
+    <t>Vifo vinavyotokana na ujauzito au kujifungua karibuni</t>
+  </si>
+  <si>
+    <t>accident</t>
+  </si>
+  <si>
+    <t>Accident</t>
+  </si>
+  <si>
+    <t>Ajali</t>
+  </si>
+  <si>
+    <t>sickness</t>
+  </si>
+  <si>
+    <t>Long-term sickness</t>
+  </si>
+  <si>
+    <t>Magonjwa ya muda mrefu</t>
+  </si>
+  <si>
+    <t>fever</t>
+  </si>
+  <si>
+    <t>Fever</t>
+  </si>
+  <si>
+    <t>Homa</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Nyenginezo</t>
+  </si>
+  <si>
+    <t>where_death</t>
+  </si>
+  <si>
+    <t>home</t>
+  </si>
+  <si>
+    <t>At home</t>
+  </si>
+  <si>
+    <t>Nyumbani</t>
+  </si>
+  <si>
+    <t>outside_home</t>
+  </si>
+  <si>
+    <t>Outside home</t>
+  </si>
+  <si>
+    <t>Nje ya nyumbani</t>
+  </si>
+  <si>
+    <t>tba</t>
+  </si>
+  <si>
+    <t>At TBA</t>
+  </si>
+  <si>
+    <t>Kwa mkunga wa jadi</t>
+  </si>
+  <si>
+    <t>health_facility</t>
+  </si>
+  <si>
+    <t>At health facility</t>
+  </si>
+  <si>
+    <t>Kwenye kituo cha afya</t>
   </si>
   <si>
     <t>user</t>
   </si>
   <si>
+    <t>Penginepo</t>
+  </si>
+  <si>
     <t>string</t>
   </si>
   <si>
@@ -138,133 +237,46 @@
     <t>Contact ID of the logged in user</t>
   </si>
   <si>
-    <t>pregnancy</t>
-  </si>
-  <si>
     <t>facility_id</t>
   </si>
   <si>
-    <t>The woman was pregnant when she died</t>
-  </si>
-  <si>
     <t>Facility ID for the parent user</t>
   </si>
   <si>
-    <t>Mama alikuwa mjamzito alipofariki</t>
-  </si>
-  <si>
-    <t>childbirth</t>
-  </si>
-  <si>
     <t>Name of the logged in user</t>
   </si>
   <si>
-    <t>The woman died during childbirth</t>
+    <t>end group</t>
+  </si>
+  <si>
+    <t>contact</t>
+  </si>
+  <si>
+    <t>date_of_birth</t>
+  </si>
+  <si>
+    <t>db:person</t>
+  </si>
+  <si>
+    <t>_id</t>
+  </si>
+  <si>
+    <t>db-object</t>
   </si>
   <si>
     <t>pages</t>
   </si>
   <si>
-    <t>Mama alifariki wakati wa kujifungua</t>
-  </si>
-  <si>
-    <t>end group</t>
-  </si>
-  <si>
     <t>data</t>
   </si>
   <si>
-    <t>after_2_3_mo</t>
-  </si>
-  <si>
-    <t>The woman died within 2 to 3 months after the end of a pregnancy or childbirth</t>
-  </si>
-  <si>
-    <t>Mama alifariki miezi miwili hadi mitatu baada ya ujauzito au baada ya kujifungua</t>
-  </si>
-  <si>
-    <t>contact</t>
-  </si>
-  <si>
-    <t>none_of_the_above</t>
-  </si>
-  <si>
-    <t>None of the above</t>
-  </si>
-  <si>
-    <t>Hakuna kati ya hizo</t>
-  </si>
-  <si>
-    <t>date_of_birth</t>
-  </si>
-  <si>
-    <t>where_death</t>
-  </si>
-  <si>
-    <t>home</t>
-  </si>
-  <si>
-    <t>At home</t>
-  </si>
-  <si>
-    <t>Nyumbani</t>
-  </si>
-  <si>
-    <t>outside_home</t>
-  </si>
-  <si>
-    <t>Outside home</t>
-  </si>
-  <si>
-    <t>db:person</t>
-  </si>
-  <si>
-    <t>Nje ya nyumbani</t>
-  </si>
-  <si>
-    <t>_id</t>
-  </si>
-  <si>
-    <t>tba</t>
-  </si>
-  <si>
-    <t>At TBA</t>
-  </si>
-  <si>
-    <t>db-object</t>
-  </si>
-  <si>
-    <t>Kwa mkunga wa jadi</t>
-  </si>
-  <si>
-    <t>other</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>Penginepo</t>
-  </si>
-  <si>
-    <t>where_pregnancy_end</t>
-  </si>
-  <si>
     <t>sex</t>
   </si>
   <si>
     <t>calculate</t>
   </si>
   <si>
-    <t>health_facility</t>
-  </si>
-  <si>
     <t>client_name</t>
-  </si>
-  <si>
-    <t>At health facility</t>
-  </si>
-  <si>
-    <t>Kwenye kituo cha afya</t>
   </si>
   <si>
     <t>../inputs/contact/name</t>
@@ -422,19 +434,19 @@
     <t>&lt;span style="color:#f58a1f"&gt;Sympathize with the family for their loss. Describe why you are asking these questions and how the information will be shared and used.&lt;/span&gt;</t>
   </si>
   <si>
-    <t>Wape pole familia kwa kufiwa na mtu wao. Waeleze kwa nini unauliza maswali haya na ni vipi hizi taarifa zitawasilishwa na kufanyiwa kazi.</t>
-  </si>
-  <si>
-    <t>select_one when_death</t>
-  </si>
-  <si>
-    <t>When did the death occur?</t>
-  </si>
-  <si>
-    <t>Kifo kilitokea lini?</t>
-  </si>
-  <si>
-    <t>${sex} = "female"</t>
+    <t>&lt;span style="color:#f58a1f"&gt;Wape pole familia kwa kufiwa na mtu wao. Waeleze kwa nini unauliza maswali haya na ni vipi hizi taarifa zitawasilishwa na kufanyiwa kazi.&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>select_one reason_death</t>
+  </si>
+  <si>
+    <t>What is the reason for the person's death?</t>
+  </si>
+  <si>
+    <t>Ni sababu ipi ilipelekea kifo cha marehemu?</t>
+  </si>
+  <si>
+    <t>${sex} = "female" and ${age_in_years} &gt;= 12</t>
   </si>
   <si>
     <t>suspected_maternal_death</t>
@@ -446,7 +458,7 @@
     <t>Utambuzi wa vifo vya akina mama</t>
   </si>
   <si>
-    <t>${sex} = "female" and ${when_death} != "none_of_the_above"</t>
+    <t>${sex} = "female" and ${age_in_years} &gt;= 12 and ${reason_death} = "pregnancy_delivery"</t>
   </si>
   <si>
     <t>date</t>
@@ -479,31 +491,37 @@
     <t>Amefia wapi</t>
   </si>
   <si>
-    <t>when_pregnancy_end</t>
-  </si>
-  <si>
-    <t>When did the pregnancy end?</t>
-  </si>
-  <si>
-    <t>Je alijifungua au mimba ilitoka lini</t>
-  </si>
-  <si>
-    <t>. &lt;= date-time(decimal-date-time(${date_of_death_maternal})) and . &gt;= date-time(decimal-date-time(${date_of_birth_c}))</t>
-  </si>
-  <si>
-    <t>The date of pregnancy loss must be between the date of birth (${date_of_birth_c}) and the date of death.</t>
-  </si>
-  <si>
-    <t>Tarehe ya kuharibika ujauzito iwe baina ya tarehe ya kifo na tarehe ya kuzaliwa</t>
-  </si>
-  <si>
-    <t>select_one where_pregnancy_end</t>
-  </si>
-  <si>
-    <t>Where did the pregnancy end?</t>
-  </si>
-  <si>
-    <t>Alijifungua au kutoka mimba wapi</t>
+    <t>select_one yes_no_dontknow</t>
+  </si>
+  <si>
+    <t>was_pregnant</t>
+  </si>
+  <si>
+    <t>Was ${client_name} pregnant when she died?</t>
+  </si>
+  <si>
+    <t>Je alipofariki alikuwa mjamzito?</t>
+  </si>
+  <si>
+    <t>select_one yes_no</t>
+  </si>
+  <si>
+    <t>during_childbirth</t>
+  </si>
+  <si>
+    <t>Did she die during childbirth?</t>
+  </si>
+  <si>
+    <t>Je alifariki wakati wa kujifungua?</t>
+  </si>
+  <si>
+    <t>two_to_three_mo_after_pregnancy_childbirth</t>
+  </si>
+  <si>
+    <t>Did she die within 2 to 3 months after the end of a pregnancy or childbirth?</t>
+  </si>
+  <si>
+    <t>Je alifariki ndani ya miezi 2-3 baada ya kujifungua au mimbakutoka?</t>
   </si>
   <si>
     <t>next_of_kin</t>
@@ -599,7 +617,7 @@
     <t>Tumia mfumo huu 0XXXXXXXXX</t>
   </si>
   <si>
-    <t>${sex} = "male" or ${when_death} = "none_of_the_above"</t>
+    <t>not(${sex} = "female" and ${age_in_years} &gt;= 12 and ${reason_death} = "pregnancy_delivery")</t>
   </si>
   <si>
     <t>date_of_death_other</t>
@@ -744,7 +762,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -756,54 +774,54 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="J1" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="K1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O1" t="s">
         <v>19</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>20</v>
       </c>
-      <c r="M1" t="s">
-        <v>21</v>
-      </c>
-      <c r="N1" t="s">
-        <v>22</v>
-      </c>
-      <c r="O1" t="s">
-        <v>23</v>
-      </c>
-      <c r="P1" t="s">
-        <v>26</v>
-      </c>
       <c r="Q1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F2" t="b">
         <f>FALSE()</f>
@@ -812,237 +830,237 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>74</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="C13" s="1"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C15" s="1"/>
       <c r="F15" s="1"/>
       <c r="L15" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C16" s="1"/>
       <c r="F16" s="1"/>
       <c r="L16" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C17" s="1"/>
       <c r="F17" s="1"/>
       <c r="L17" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C18" s="1"/>
       <c r="F18" s="1"/>
       <c r="L18" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="5"/>
@@ -1054,7 +1072,7 @@
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
       <c r="L22" s="6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="M22" s="7"/>
       <c r="N22" s="7"/>
@@ -1073,10 +1091,10 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="5"/>
@@ -1088,7 +1106,7 @@
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
       <c r="L23" s="9" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="M23" s="7"/>
       <c r="N23" s="5"/>
@@ -1107,10 +1125,10 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="5"/>
@@ -1122,7 +1140,7 @@
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>
       <c r="L24" s="9" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="M24" s="5"/>
       <c r="N24" s="5"/>
@@ -1141,10 +1159,10 @@
     </row>
     <row r="25">
       <c r="A25" s="8" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C25" s="4"/>
       <c r="D25" s="5"/>
@@ -1156,7 +1174,7 @@
       <c r="J25" s="5"/>
       <c r="K25" s="5"/>
       <c r="L25" s="10" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="R25" s="5"/>
       <c r="S25" s="5"/>
@@ -1170,10 +1188,10 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="5"/>
@@ -1185,7 +1203,7 @@
       <c r="J26" s="5"/>
       <c r="K26" s="5"/>
       <c r="L26" s="9" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M26" s="7"/>
       <c r="N26" s="5"/>
@@ -1204,77 +1222,77 @@
     </row>
     <row r="27">
       <c r="A27" s="11" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C27" s="2"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="L27" s="12" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C28" s="2"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="L28" s="12" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C29" s="2"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="L29" s="12" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C30" s="2"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="L30" s="12" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E31" s="5"/>
       <c r="F31" s="13"/>
       <c r="G31" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
@@ -1298,16 +1316,16 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="E32" s="7"/>
       <c r="F32" s="4"/>
@@ -1334,16 +1352,16 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E33" s="7"/>
       <c r="F33" s="4"/>
@@ -1370,16 +1388,16 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E34" s="5"/>
       <c r="F34" s="4"/>
@@ -1406,10 +1424,10 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C35" s="4"/>
       <c r="D35" s="5"/>
@@ -1438,13 +1456,13 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D36" s="5"/>
       <c r="F36" s="1"/>
@@ -1452,16 +1470,16 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>133</v>
+        <v>136</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>137</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" s="1"/>
@@ -1470,32 +1488,32 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>136</v>
+        <v>139</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>140</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="G38" s="1"/>
       <c r="L38" s="1"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -1508,23 +1526,23 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" s="2" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
@@ -1532,45 +1550,45 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G42" s="1"/>
       <c r="I42" s="2"/>
@@ -1579,124 +1597,112 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G43" s="1"/>
-      <c r="I43" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>157</v>
-      </c>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
       <c r="L43" s="1"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>77</v>
+        <v>161</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G44" s="1"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
       <c r="L44" s="1"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>51</v>
+        <v>160</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="G45" s="2"/>
+        <v>164</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G45" s="1"/>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
       <c r="L45" s="1"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>163</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
       <c r="E46" s="2"/>
-      <c r="F46" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>119</v>
-      </c>
+      <c r="G46" s="2"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="L46" s="1"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F47" s="2"/>
-      <c r="G47" s="1"/>
-      <c r="I47" s="17" t="s">
-        <v>167</v>
-      </c>
-      <c r="J47" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="K47" s="18" t="s">
         <v>169</v>
       </c>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="I47" s="2"/>
+      <c r="J47" s="2"/>
       <c r="L47" s="1"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>170</v>
@@ -1708,174 +1714,203 @@
         <v>172</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F48" s="2"/>
       <c r="G48" s="1"/>
       <c r="I48" s="17" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="J48" s="18" t="s">
-        <v>173</v>
-      </c>
-      <c r="K48" s="2" t="s">
         <v>174</v>
+      </c>
+      <c r="K48" s="18" t="s">
+        <v>175</v>
       </c>
       <c r="L48" s="1"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F49" s="2"/>
       <c r="G49" s="1"/>
       <c r="I49" s="17" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="J49" s="18" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L49" s="1"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F50" s="2"/>
       <c r="G50" s="1"/>
       <c r="I50" s="17" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="J50" s="18" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="L50" s="1"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F51" s="2"/>
-      <c r="G51" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="I51" s="2" t="s">
+      <c r="G51" s="1"/>
+      <c r="I51" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="J51" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="J51" s="11" t="s">
+      <c r="K51" s="2" t="s">
         <v>190</v>
-      </c>
-      <c r="K51" s="18" t="s">
-        <v>191</v>
       </c>
       <c r="L51" s="1"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C52" s="2"/>
-      <c r="E52" s="2"/>
+        <v>191</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="F52" s="2"/>
-      <c r="G52" s="1"/>
-      <c r="I52" s="2"/>
-      <c r="J52" s="2"/>
+      <c r="G52" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="J52" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="K52" s="18" t="s">
+        <v>197</v>
+      </c>
       <c r="L52" s="1"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>119</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="C53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="1"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="2"/>
+      <c r="L53" s="1"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="s">
-        <v>142</v>
+        <v>34</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>193</v>
+        <v>53</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="I54" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="J54" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="K54" s="2" t="s">
-        <v>148</v>
+        <v>36</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="s">
-        <v>51</v>
+        <v>146</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>74</v>
+        <v>199</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1899,7 +1934,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1913,198 +1948,212 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>43</v>
+        <v>32</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>48</v>
+        <v>32</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D6" t="s">
-        <v>55</v>
+        <v>38</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" t="s">
-        <v>59</v>
+        <v>42</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>83</v>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -2121,40 +2170,40 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E1" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C2" s="3" t="str">
         <f>TEXT(NOW(), "yyyy-mm-dd_HH-MM")</f>
-        <v>2019-09-27_15-55</v>
+        <v>2019-10-24_11-11</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>83</v>
       </c>
       <c r="E2" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Covid-19 Form Messages (#131)
* Added Covid19 Message for CHVs in all forms which has interactions between CHVs and clients
</commit_message>
<xml_diff>
--- a/forms/app/death_report.xlsx
+++ b/forms/app/death_report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="208">
   <si>
     <t>list_name</t>
   </si>
@@ -42,9 +42,18 @@
     <t>version</t>
   </si>
   <si>
+    <t>style</t>
+  </si>
+  <si>
     <t>required</t>
   </si>
   <si>
+    <t>path</t>
+  </si>
+  <si>
+    <t>instance_name</t>
+  </si>
+  <si>
     <t>relevant</t>
   </si>
   <si>
@@ -72,33 +81,36 @@
     <t>hint::en</t>
   </si>
   <si>
+    <t>Death Report</t>
+  </si>
+  <si>
     <t>hint::sw</t>
   </si>
   <si>
     <t>default</t>
   </si>
   <si>
-    <t>style</t>
+    <t>repeat_count</t>
+  </si>
+  <si>
+    <t>begin group</t>
+  </si>
+  <si>
+    <t>inputs</t>
+  </si>
+  <si>
+    <t>NO_LABEL</t>
   </si>
   <si>
     <t>yes</t>
   </si>
   <si>
-    <t>path</t>
-  </si>
-  <si>
-    <t>instance_name</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
     <t>Ndiyo</t>
   </si>
   <si>
-    <t>Death Report</t>
-  </si>
-  <si>
     <t>death_report</t>
   </si>
   <si>
@@ -108,22 +120,52 @@
     <t>No</t>
   </si>
   <si>
+    <t>user</t>
+  </si>
+  <si>
     <t>Hapana</t>
   </si>
   <si>
     <t>yes_no_dontknow</t>
   </si>
   <si>
-    <t>repeat_count</t>
-  </si>
-  <si>
-    <t>begin group</t>
-  </si>
-  <si>
-    <t>inputs</t>
-  </si>
-  <si>
-    <t>NO_LABEL</t>
+    <t>string</t>
+  </si>
+  <si>
+    <t>contact_id</t>
+  </si>
+  <si>
+    <t>Contact ID of the logged in user</t>
+  </si>
+  <si>
+    <t>facility_id</t>
+  </si>
+  <si>
+    <t>Facility ID for the parent user</t>
+  </si>
+  <si>
+    <t>Name of the logged in user</t>
+  </si>
+  <si>
+    <t>end group</t>
+  </si>
+  <si>
+    <t>contact</t>
+  </si>
+  <si>
+    <t>date_of_birth</t>
+  </si>
+  <si>
+    <t>db:person</t>
+  </si>
+  <si>
+    <t>_id</t>
+  </si>
+  <si>
+    <t>db-object</t>
+  </si>
+  <si>
+    <t>sex</t>
   </si>
   <si>
     <t>dont_know</t>
@@ -135,18 +177,33 @@
     <t>Sijui</t>
   </si>
   <si>
+    <t>pages</t>
+  </si>
+  <si>
     <t>reason_death</t>
   </si>
   <si>
+    <t>data</t>
+  </si>
+  <si>
+    <t>calculate</t>
+  </si>
+  <si>
     <t>pregnancy_delivery</t>
   </si>
   <si>
+    <t>client_name</t>
+  </si>
+  <si>
     <t>Death related to pregnancy or recent delivery</t>
   </si>
   <si>
     <t>Vifo vinavyotokana na ujauzito au kujifungua karibuni</t>
   </si>
   <si>
+    <t>../inputs/contact/name</t>
+  </si>
+  <si>
     <t>accident</t>
   </si>
   <si>
@@ -156,15 +213,24 @@
     <t>Ajali</t>
   </si>
   <si>
+    <t>patient_id</t>
+  </si>
+  <si>
     <t>sickness</t>
   </si>
   <si>
+    <t>../inputs/contact/_id</t>
+  </si>
+  <si>
     <t>Long-term sickness</t>
   </si>
   <si>
     <t>Magonjwa ya muda mrefu</t>
   </si>
   <si>
+    <t>date_of_birth_c</t>
+  </si>
+  <si>
     <t>fever</t>
   </si>
   <si>
@@ -174,6 +240,9 @@
     <t>Homa</t>
   </si>
   <si>
+    <t>../inputs/contact/date_of_birth</t>
+  </si>
+  <si>
     <t>other</t>
   </si>
   <si>
@@ -183,27 +252,42 @@
     <t>Nyenginezo</t>
   </si>
   <si>
+    <t>sex_c</t>
+  </si>
+  <si>
     <t>where_death</t>
   </si>
   <si>
     <t>home</t>
   </si>
   <si>
+    <t>../inputs/contact/sex</t>
+  </si>
+  <si>
     <t>At home</t>
   </si>
   <si>
     <t>Nyumbani</t>
   </si>
   <si>
+    <t>created_by</t>
+  </si>
+  <si>
     <t>outside_home</t>
   </si>
   <si>
     <t>Outside home</t>
   </si>
   <si>
+    <t>hidden</t>
+  </si>
+  <si>
     <t>Nje ya nyumbani</t>
   </si>
   <si>
+    <t>../inputs/user/name</t>
+  </si>
+  <si>
     <t>tba</t>
   </si>
   <si>
@@ -213,111 +297,27 @@
     <t>Kwa mkunga wa jadi</t>
   </si>
   <si>
+    <t>created_by_person_uuid</t>
+  </si>
+  <si>
     <t>health_facility</t>
   </si>
   <si>
+    <t>../inputs/user/contact_id</t>
+  </si>
+  <si>
     <t>At health facility</t>
   </si>
   <si>
     <t>Kwenye kituo cha afya</t>
   </si>
   <si>
-    <t>user</t>
+    <t>created_by_place_uuid</t>
   </si>
   <si>
     <t>Penginepo</t>
   </si>
   <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>contact_id</t>
-  </si>
-  <si>
-    <t>Contact ID of the logged in user</t>
-  </si>
-  <si>
-    <t>facility_id</t>
-  </si>
-  <si>
-    <t>Facility ID for the parent user</t>
-  </si>
-  <si>
-    <t>Name of the logged in user</t>
-  </si>
-  <si>
-    <t>end group</t>
-  </si>
-  <si>
-    <t>contact</t>
-  </si>
-  <si>
-    <t>date_of_birth</t>
-  </si>
-  <si>
-    <t>db:person</t>
-  </si>
-  <si>
-    <t>_id</t>
-  </si>
-  <si>
-    <t>db-object</t>
-  </si>
-  <si>
-    <t>pages</t>
-  </si>
-  <si>
-    <t>data</t>
-  </si>
-  <si>
-    <t>sex</t>
-  </si>
-  <si>
-    <t>calculate</t>
-  </si>
-  <si>
-    <t>client_name</t>
-  </si>
-  <si>
-    <t>../inputs/contact/name</t>
-  </si>
-  <si>
-    <t>patient_id</t>
-  </si>
-  <si>
-    <t>../inputs/contact/_id</t>
-  </si>
-  <si>
-    <t>date_of_birth_c</t>
-  </si>
-  <si>
-    <t>../inputs/contact/date_of_birth</t>
-  </si>
-  <si>
-    <t>sex_c</t>
-  </si>
-  <si>
-    <t>../inputs/contact/sex</t>
-  </si>
-  <si>
-    <t>created_by</t>
-  </si>
-  <si>
-    <t>hidden</t>
-  </si>
-  <si>
-    <t>../inputs/user/name</t>
-  </si>
-  <si>
-    <t>created_by_person_uuid</t>
-  </si>
-  <si>
-    <t>../inputs/user/contact_id</t>
-  </si>
-  <si>
-    <t>created_by_place_uuid</t>
-  </si>
-  <si>
     <t>../inputs/user/facility_id</t>
   </si>
   <si>
@@ -375,6 +375,49 @@
     <t>instance('contact-summary')/context/phone</t>
   </si>
   <si>
+    <t xml:space="preserve">begin group </t>
+  </si>
+  <si>
+    <t>covid19_intro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precautionary measures when visiting a client  </t>
+  </si>
+  <si>
+    <t>Hatua za kuchukua pindi unapoenda kumtembelea mteja wako</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>covid19_intro_note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;span style="color:#f58a1f"&gt;As a CHV, you are responsible for making sure that you are providing the community with health education and services while trying to take precautions to stop the transmission of Corona virus to one another. Therefore, make sure you consider the following while you conduct the visits:  
+•        Wash your hands with soap/sanitizer as many time as you can while at home, once you are at the client’s house and when you leave.
+•        Keep a 2 meters distance while talking to your clients.
+•        Don’t shake hands with your clients. 
+•        Avoid group gatherings.
+•        Provide the service at the open space and if it should be inside, make sure the windows and doors are open. 
+•        Cover your mouth with a towel or elbow when you sneeze or cough. 
+•        Do not go for a visit if you have symptoms of fever, cough or frequent sneezing.&lt;/span&gt; 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;span style="color:#f58a1f"&gt;Kama mhudumu wa afya ya jamii, una jukumu la kuhakikisha unatoa elimu ya afya ya jamii na huduma huku ukijikinga ili kuepusha kusambaa kwa maambukizi ya korona kutoka kwa mtu mmoja kwenda kwa mwengine. Hivyo hakikisha unazingatia yafuatayo wakati ukiwa unatoa huduma:
+•        Osha mikono yako kwa maji na sabuni au kutumia vitakasa mikono mara nyingi kadiri unavyoweza ukiwa nyumbani kwako,nyumbani kwa mteja wako na pindi ukimaliza kutoa huduma. 
+•        Hakikisha kuna umbali wa mita mbili kati yako na mteja wako unayeenda kumtembelea 
+•        Pindi ukiongea na wateja wako , usishikane mikono. 
+•        Epuka mikusanyiko. 
+•        Toa huduma katika maeneo yaliyo wazi na ikitokea ukafanya ndani hakikisha milango na madirisha yanakuwa wazi.  
+•        Funika mdomo wako kwa kitambaa au kiwiko unavyooenda chafya au kukohoa. 
+•        Tafadhali usiende kutoa huduma ukijihisi na dalili za homa na kukohoa na kwenda chafya kwa wingi.&lt;/span&gt; 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">end group </t>
+  </si>
+  <si>
     <t>client_information</t>
   </si>
   <si>
@@ -385,9 +428,6 @@
   </si>
   <si>
     <t>field-list</t>
-  </si>
-  <si>
-    <t>note</t>
   </si>
   <si>
     <t>intro_note</t>
@@ -627,7 +667,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -646,12 +686,16 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF1D1C1D"/>
+      <name val="Slack-Lato"/>
+    </font>
+    <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Sans"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -664,6 +708,12 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8F8F8"/>
+        <bgColor rgb="FFF8F8F8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -674,7 +724,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -710,6 +760,15 @@
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
@@ -722,7 +781,7 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
@@ -774,54 +833,54 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="J1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="K1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="L1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="M1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="N1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="O1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="P1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="Q1" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="F2" t="b">
         <f>FALSE()</f>
@@ -830,226 +889,226 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>73</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>81</v>
+        <v>48</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="G10" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="C13" s="1"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="C15" s="1"/>
       <c r="F15" s="1"/>
       <c r="L15" s="1" t="s">
-        <v>88</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C16" s="1"/>
       <c r="F16" s="1"/>
       <c r="L16" s="1" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="C17" s="1"/>
       <c r="F17" s="1"/>
       <c r="L17" s="1" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="C18" s="1"/>
       <c r="F18" s="1"/>
       <c r="L18" s="2" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="C19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L20" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="L21" s="1" t="s">
         <v>101</v>
@@ -1057,7 +1116,7 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>102</v>
@@ -1091,7 +1150,7 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>104</v>
@@ -1125,7 +1184,7 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B24" s="8" t="s">
         <v>106</v>
@@ -1159,7 +1218,7 @@
     </row>
     <row r="25">
       <c r="A25" s="8" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>108</v>
@@ -1188,7 +1247,7 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>110</v>
@@ -1222,7 +1281,7 @@
     </row>
     <row r="27">
       <c r="A27" s="11" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>112</v>
@@ -1236,7 +1295,7 @@
     </row>
     <row r="28">
       <c r="A28" s="11" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>114</v>
@@ -1250,7 +1309,7 @@
     </row>
     <row r="29">
       <c r="A29" s="11" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>116</v>
@@ -1264,7 +1323,7 @@
     </row>
     <row r="30">
       <c r="A30" s="11" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>118</v>
@@ -1277,131 +1336,106 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B31" s="4" t="s">
+      <c r="A31" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="B31" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="C31" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="E31" s="5"/>
+      <c r="D31" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="E31" s="15"/>
       <c r="F31" s="13"/>
-      <c r="G31" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
-      <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
-      <c r="L31" s="4"/>
-      <c r="M31" s="5"/>
-      <c r="N31" s="5"/>
-      <c r="O31" s="5"/>
-      <c r="P31" s="5"/>
-      <c r="Q31" s="5"/>
-      <c r="R31" s="5"/>
-      <c r="S31" s="5"/>
-      <c r="T31" s="5"/>
-      <c r="U31" s="5"/>
-      <c r="V31" s="5"/>
-      <c r="W31" s="5"/>
-      <c r="X31" s="5"/>
-      <c r="Y31" s="5"/>
-      <c r="Z31" s="5"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="15"/>
+      <c r="I31" s="15"/>
+      <c r="J31" s="15"/>
+      <c r="K31" s="15"/>
+      <c r="L31" s="13"/>
+      <c r="M31" s="15"/>
+      <c r="N31" s="15"/>
+      <c r="O31" s="15"/>
+      <c r="P31" s="15"/>
+      <c r="Q31" s="15"/>
+      <c r="R31" s="15"/>
+      <c r="S31" s="15"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="C32" s="14" t="s">
+      <c r="C32" s="13" t="s">
         <v>126</v>
       </c>
       <c r="D32" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="E32" s="7"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
-      <c r="L32" s="4"/>
-      <c r="M32" s="5"/>
-      <c r="N32" s="5"/>
-      <c r="O32" s="5"/>
-      <c r="P32" s="5"/>
-      <c r="Q32" s="5"/>
-      <c r="R32" s="5"/>
-      <c r="S32" s="5"/>
-      <c r="T32" s="5"/>
-      <c r="U32" s="5"/>
-      <c r="V32" s="5"/>
-      <c r="W32" s="5"/>
-      <c r="X32" s="5"/>
-      <c r="Y32" s="5"/>
-      <c r="Z32" s="5"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="15"/>
+      <c r="K32" s="15"/>
+      <c r="L32" s="13"/>
+      <c r="M32" s="15"/>
+      <c r="N32" s="15"/>
+      <c r="O32" s="15"/>
+      <c r="P32" s="15"/>
+      <c r="Q32" s="15"/>
+      <c r="R32" s="15"/>
+      <c r="S32" s="15"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="B33" s="4" t="s">
+      <c r="A33" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="C33" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="E33" s="7"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
-      <c r="L33" s="4"/>
-      <c r="M33" s="5"/>
-      <c r="N33" s="5"/>
-      <c r="O33" s="5"/>
-      <c r="P33" s="5"/>
-      <c r="Q33" s="5"/>
-      <c r="R33" s="5"/>
-      <c r="S33" s="5"/>
-      <c r="T33" s="5"/>
-      <c r="U33" s="5"/>
-      <c r="V33" s="5"/>
-      <c r="W33" s="5"/>
-      <c r="X33" s="5"/>
-      <c r="Y33" s="5"/>
-      <c r="Z33" s="5"/>
+      <c r="B33" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C33" s="13"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="15"/>
+      <c r="J33" s="15"/>
+      <c r="K33" s="15"/>
+      <c r="L33" s="13"/>
+      <c r="M33" s="15"/>
+      <c r="N33" s="15"/>
+      <c r="O33" s="15"/>
+      <c r="P33" s="15"/>
+      <c r="Q33" s="15"/>
+      <c r="R33" s="15"/>
+      <c r="S33" s="15"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="s">
-        <v>124</v>
+        <v>26</v>
       </c>
       <c r="B34" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="E34" s="5"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="D34" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="E34" s="5"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
@@ -1424,14 +1458,18 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="s">
-        <v>77</v>
+        <v>124</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
+        <v>133</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="E35" s="7"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="5"/>
@@ -1455,97 +1493,139 @@
       <c r="Z35" s="5"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D36" s="5"/>
-      <c r="F36" s="1"/>
-      <c r="L36" s="1"/>
+      <c r="A36" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="E36" s="7"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="5"/>
+      <c r="N36" s="5"/>
+      <c r="O36" s="5"/>
+      <c r="P36" s="5"/>
+      <c r="Q36" s="5"/>
+      <c r="R36" s="5"/>
+      <c r="S36" s="5"/>
+      <c r="T36" s="5"/>
+      <c r="U36" s="5"/>
+      <c r="V36" s="5"/>
+      <c r="W36" s="5"/>
+      <c r="X36" s="5"/>
+      <c r="Y36" s="5"/>
+      <c r="Z36" s="5"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="s">
+      <c r="A37" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="D37" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="E37" s="2"/>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="L37" s="1"/>
+      <c r="B37" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D37" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="E37" s="5"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="5"/>
+      <c r="N37" s="5"/>
+      <c r="O37" s="5"/>
+      <c r="P37" s="5"/>
+      <c r="Q37" s="5"/>
+      <c r="R37" s="5"/>
+      <c r="S37" s="5"/>
+      <c r="T37" s="5"/>
+      <c r="U37" s="5"/>
+      <c r="V37" s="5"/>
+      <c r="W37" s="5"/>
+      <c r="X37" s="5"/>
+      <c r="Y37" s="5"/>
+      <c r="Z37" s="5"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="D38" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="G38" s="1"/>
-      <c r="L38" s="1"/>
+      <c r="A38" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C38" s="4"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="5"/>
+      <c r="L38" s="4"/>
+      <c r="M38" s="5"/>
+      <c r="N38" s="5"/>
+      <c r="O38" s="5"/>
+      <c r="P38" s="5"/>
+      <c r="Q38" s="5"/>
+      <c r="R38" s="5"/>
+      <c r="S38" s="5"/>
+      <c r="T38" s="5"/>
+      <c r="U38" s="5"/>
+      <c r="V38" s="5"/>
+      <c r="W38" s="5"/>
+      <c r="X38" s="5"/>
+      <c r="Y38" s="5"/>
+      <c r="Z38" s="5"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>77</v>
+        <v>26</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-      <c r="I39" s="2"/>
-      <c r="J39" s="2"/>
+        <v>142</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D39" s="5"/>
+      <c r="F39" s="1"/>
       <c r="L39" s="1"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>34</v>
+        <v>124</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D40" s="2" t="s">
         <v>144</v>
       </c>
+      <c r="D40" s="17" t="s">
+        <v>145</v>
+      </c>
       <c r="E40" s="2"/>
-      <c r="F40" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
       <c r="L40" s="1"/>
     </row>
     <row r="41">
@@ -1553,364 +1633,426 @@
         <v>146</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="D41" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="E41" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E41" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>152</v>
-      </c>
+      <c r="G41" s="1"/>
+      <c r="L41" s="1"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>153</v>
+        <v>44</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G42" s="1"/>
+        <v>142</v>
+      </c>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="L42" s="1"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>156</v>
+        <v>26</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G43" s="1"/>
+        <v>152</v>
+      </c>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>132</v>
+      </c>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
-      <c r="K43" s="2"/>
       <c r="L43" s="1"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="K44" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G44" s="1"/>
-      <c r="I44" s="2"/>
-      <c r="J44" s="2"/>
-      <c r="K44" s="2"/>
-      <c r="L44" s="1"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>164</v>
+        <v>80</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="G45" s="1"/>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
       <c r="L45" s="1"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>77</v>
+        <v>164</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="G46" s="2"/>
+        <v>165</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G46" s="1"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
       <c r="L46" s="1"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>34</v>
+        <v>168</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>123</v>
-      </c>
+        <v>171</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G47" s="1"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
       <c r="L47" s="1"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>71</v>
+        <v>168</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F48" s="2"/>
+        <v>29</v>
+      </c>
       <c r="G48" s="1"/>
-      <c r="I48" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="J48" s="18" t="s">
-        <v>174</v>
-      </c>
-      <c r="K48" s="18" t="s">
-        <v>175</v>
-      </c>
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2"/>
       <c r="L48" s="1"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F49" s="2"/>
-      <c r="G49" s="1"/>
-      <c r="I49" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="J49" s="18" t="s">
-        <v>179</v>
-      </c>
-      <c r="K49" s="2" t="s">
-        <v>180</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="G49" s="2"/>
+      <c r="I49" s="2"/>
+      <c r="J49" s="2"/>
       <c r="L49" s="1"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="s">
-        <v>71</v>
+        <v>26</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F50" s="2"/>
-      <c r="G50" s="1"/>
-      <c r="I50" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="J50" s="18" t="s">
-        <v>184</v>
-      </c>
-      <c r="K50" s="2" t="s">
-        <v>185</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="E50" s="2"/>
+      <c r="F50" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="I50" s="2"/>
+      <c r="J50" s="2"/>
       <c r="L50" s="1"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F51" s="2"/>
       <c r="G51" s="1"/>
-      <c r="I51" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="J51" s="18" t="s">
-        <v>189</v>
-      </c>
-      <c r="K51" s="2" t="s">
-        <v>190</v>
+      <c r="I51" s="20" t="s">
+        <v>181</v>
+      </c>
+      <c r="J51" s="21" t="s">
+        <v>182</v>
+      </c>
+      <c r="K51" s="21" t="s">
+        <v>183</v>
       </c>
       <c r="L51" s="1"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F52" s="2"/>
-      <c r="G52" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="I52" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="J52" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="K52" s="18" t="s">
-        <v>197</v>
+      <c r="G52" s="1"/>
+      <c r="I52" s="20" t="s">
+        <v>181</v>
+      </c>
+      <c r="J52" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>188</v>
       </c>
       <c r="L52" s="1"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="s">
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="C53" s="2"/>
-      <c r="E53" s="2"/>
+        <v>189</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="F53" s="2"/>
       <c r="G53" s="1"/>
-      <c r="I53" s="2"/>
-      <c r="J53" s="2"/>
+      <c r="I53" s="20" t="s">
+        <v>181</v>
+      </c>
+      <c r="J53" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>193</v>
+      </c>
       <c r="L53" s="1"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>53</v>
+        <v>194</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F54" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F54" s="2"/>
+      <c r="G54" s="1"/>
+      <c r="I54" s="20" t="s">
+        <v>181</v>
+      </c>
+      <c r="J54" s="21" t="s">
+        <v>197</v>
+      </c>
+      <c r="K54" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="G54" s="2" t="s">
-        <v>123</v>
-      </c>
+      <c r="L54" s="1"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="s">
-        <v>146</v>
+        <v>38</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>199</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>148</v>
+        <v>200</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>149</v>
+        <v>201</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>22</v>
+        <v>29</v>
+      </c>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2" t="s">
+        <v>202</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="J55" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="K55" s="2" t="s">
-        <v>152</v>
-      </c>
+        <v>203</v>
+      </c>
+      <c r="J55" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="K55" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="L55" s="1"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>53</v>
+        <v>175</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="1"/>
+      <c r="I56" s="2"/>
+      <c r="J56" s="2"/>
+      <c r="L56" s="1"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1928,6 +2070,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
   <cols>
+    <col customWidth="1" min="1" max="1" width="35.57"/>
     <col customWidth="1" min="2" max="2" width="18.29"/>
     <col customWidth="1" min="3" max="3" width="33.14"/>
   </cols>
@@ -1951,13 +2094,13 @@
         <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -1965,195 +2108,195 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>62</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>65</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>66</v>
+        <v>95</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2179,31 +2322,31 @@
         <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="F1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C2" s="3" t="str">
         <f>TEXT(NOW(), "yyyy-mm-dd_HH-MM")</f>
-        <v>2019-10-24_11-11</v>
+        <v>2020-04-15_12-02</v>
       </c>
       <c r="D2" t="s">
-        <v>83</v>
+        <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Covid education protocol (#137)
* Created covid education form

* Adding reminder message for chv to perform corona visits

* removed the condition which restrict choosing the listed questions with other options

* moved the form to household and addressed the grammer errors

Co-authored-by: nitusima <nkataraia@d-treee.org>
</commit_message>
<xml_diff>
--- a/forms/app/death_report.xlsx
+++ b/forms/app/death_report.xlsx
@@ -30,36 +30,36 @@
     <t>yes_no</t>
   </si>
   <si>
+    <t>form_title</t>
+  </si>
+  <si>
     <t>type</t>
   </si>
   <si>
-    <t>form_title</t>
-  </si>
-  <si>
     <t>form_id</t>
   </si>
   <si>
     <t>version</t>
   </si>
   <si>
+    <t>required</t>
+  </si>
+  <si>
     <t>style</t>
   </si>
   <si>
-    <t>required</t>
+    <t>relevant</t>
   </si>
   <si>
     <t>path</t>
   </si>
   <si>
+    <t>appearance</t>
+  </si>
+  <si>
     <t>instance_name</t>
   </si>
   <si>
-    <t>relevant</t>
-  </si>
-  <si>
-    <t>appearance</t>
-  </si>
-  <si>
     <t>read_only</t>
   </si>
   <si>
@@ -75,15 +75,15 @@
     <t>calculation</t>
   </si>
   <si>
+    <t>Death Report</t>
+  </si>
+  <si>
     <t>choice_filter</t>
   </si>
   <si>
     <t>hint::en</t>
   </si>
   <si>
-    <t>Death Report</t>
-  </si>
-  <si>
     <t>hint::sw</t>
   </si>
   <si>
@@ -102,42 +102,42 @@
     <t>NO_LABEL</t>
   </si>
   <si>
+    <t>user</t>
+  </si>
+  <si>
     <t>yes</t>
   </si>
   <si>
+    <t>death_report</t>
+  </si>
+  <si>
     <t>Yes</t>
   </si>
   <si>
     <t>Ndiyo</t>
   </si>
   <si>
-    <t>death_report</t>
+    <t>string</t>
+  </si>
+  <si>
+    <t>contact_id</t>
   </si>
   <si>
     <t>no</t>
   </si>
   <si>
+    <t>Contact ID of the logged in user</t>
+  </si>
+  <si>
     <t>No</t>
   </si>
   <si>
-    <t>user</t>
-  </si>
-  <si>
     <t>Hapana</t>
   </si>
   <si>
     <t>yes_no_dontknow</t>
   </si>
   <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>contact_id</t>
-  </si>
-  <si>
-    <t>Contact ID of the logged in user</t>
-  </si>
-  <si>
     <t>facility_id</t>
   </si>
   <si>
@@ -159,81 +159,81 @@
     <t>db:person</t>
   </si>
   <si>
+    <t>dont_know</t>
+  </si>
+  <si>
     <t>_id</t>
   </si>
   <si>
+    <t>I don't know</t>
+  </si>
+  <si>
+    <t>Sijui</t>
+  </si>
+  <si>
+    <t>pages</t>
+  </si>
+  <si>
+    <t>reason_death</t>
+  </si>
+  <si>
     <t>db-object</t>
   </si>
   <si>
+    <t>pregnancy_delivery</t>
+  </si>
+  <si>
+    <t>Death related to pregnancy or recent delivery</t>
+  </si>
+  <si>
+    <t>data</t>
+  </si>
+  <si>
+    <t>Vifo vinavyotokana na ujauzito au kujifungua karibuni</t>
+  </si>
+  <si>
     <t>sex</t>
   </si>
   <si>
-    <t>dont_know</t>
-  </si>
-  <si>
-    <t>I don't know</t>
-  </si>
-  <si>
-    <t>Sijui</t>
-  </si>
-  <si>
-    <t>pages</t>
-  </si>
-  <si>
-    <t>reason_death</t>
-  </si>
-  <si>
-    <t>data</t>
+    <t>accident</t>
   </si>
   <si>
     <t>calculate</t>
   </si>
   <si>
-    <t>pregnancy_delivery</t>
+    <t>Accident</t>
+  </si>
+  <si>
+    <t>Ajali</t>
   </si>
   <si>
     <t>client_name</t>
   </si>
   <si>
-    <t>Death related to pregnancy or recent delivery</t>
-  </si>
-  <si>
-    <t>Vifo vinavyotokana na ujauzito au kujifungua karibuni</t>
-  </si>
-  <si>
     <t>../inputs/contact/name</t>
   </si>
   <si>
-    <t>accident</t>
-  </si>
-  <si>
-    <t>Accident</t>
-  </si>
-  <si>
-    <t>Ajali</t>
+    <t>sickness</t>
+  </si>
+  <si>
+    <t>Long-term sickness</t>
   </si>
   <si>
     <t>patient_id</t>
   </si>
   <si>
-    <t>sickness</t>
+    <t>Magonjwa ya muda mrefu</t>
   </si>
   <si>
     <t>../inputs/contact/_id</t>
   </si>
   <si>
-    <t>Long-term sickness</t>
-  </si>
-  <si>
-    <t>Magonjwa ya muda mrefu</t>
+    <t>fever</t>
   </si>
   <si>
     <t>date_of_birth_c</t>
   </si>
   <si>
-    <t>fever</t>
-  </si>
-  <si>
     <t>Fever</t>
   </si>
   <si>
@@ -246,31 +246,40 @@
     <t>other</t>
   </si>
   <si>
+    <t>sex_c</t>
+  </si>
+  <si>
     <t>Other</t>
   </si>
   <si>
+    <t>../inputs/contact/sex</t>
+  </si>
+  <si>
     <t>Nyenginezo</t>
   </si>
   <si>
-    <t>sex_c</t>
-  </si>
-  <si>
     <t>where_death</t>
   </si>
   <si>
+    <t>created_by</t>
+  </si>
+  <si>
     <t>home</t>
   </si>
   <si>
-    <t>../inputs/contact/sex</t>
-  </si>
-  <si>
     <t>At home</t>
   </si>
   <si>
+    <t>hidden</t>
+  </si>
+  <si>
     <t>Nyumbani</t>
   </si>
   <si>
-    <t>created_by</t>
+    <t>../inputs/user/name</t>
+  </si>
+  <si>
+    <t>created_by_person_uuid</t>
   </si>
   <si>
     <t>outside_home</t>
@@ -279,46 +288,37 @@
     <t>Outside home</t>
   </si>
   <si>
-    <t>hidden</t>
+    <t>../inputs/user/contact_id</t>
   </si>
   <si>
     <t>Nje ya nyumbani</t>
   </si>
   <si>
-    <t>../inputs/user/name</t>
+    <t>created_by_place_uuid</t>
   </si>
   <si>
     <t>tba</t>
   </si>
   <si>
+    <t>../inputs/user/facility_id</t>
+  </si>
+  <si>
     <t>At TBA</t>
   </si>
   <si>
     <t>Kwa mkunga wa jadi</t>
   </si>
   <si>
-    <t>created_by_person_uuid</t>
-  </si>
-  <si>
     <t>health_facility</t>
   </si>
   <si>
-    <t>../inputs/user/contact_id</t>
-  </si>
-  <si>
     <t>At health facility</t>
   </si>
   <si>
     <t>Kwenye kituo cha afya</t>
   </si>
   <si>
-    <t>created_by_place_uuid</t>
-  </si>
-  <si>
     <t>Penginepo</t>
-  </si>
-  <si>
-    <t>../inputs/user/facility_id</t>
   </si>
   <si>
     <t>age_days</t>
@@ -400,7 +400,8 @@
 •        Avoid group gatherings.
 •        Provide the service at the open space and if it should be inside, make sure the windows and doors are open. 
 •        Cover your mouth with a towel or elbow when you sneeze or cough. 
-•        Do not go for a visit if you have symptoms of fever, cough or frequent sneezing.&lt;/span&gt; 
+•        Do not go for a visit if you have symptoms of fever, cough or frequent sneezing.
+•        Please remember to do the covid education visit before or after submitting this form. &lt;/span&gt; 
 </t>
   </si>
   <si>
@@ -411,7 +412,8 @@
 •        Epuka mikusanyiko. 
 •        Toa huduma katika maeneo yaliyo wazi na ikitokea ukafanya ndani hakikisha milango na madirisha yanakuwa wazi.  
 •        Funika mdomo wako kwa kitambaa au kiwiko unavyooenda chafya au kukohoa. 
-•        Tafadhali usiende kutoa huduma ukijihisi na dalili za homa na kukohoa na kwenda chafya kwa wingi.&lt;/span&gt; 
+•        Tafadhali usiende kutoa huduma ukijihisi na dalili za homa na kukohoa na kwenda chafya kwa wingi.
+•        Tafadhali kumbuka kufungua fomu ya kuwaelimsiha wanakaya juu ya maambukizi ya korona na jinsi ya kuchukua tahadhari. Tembeleo kuhusu korona unaweza kulifanya kabla ya kuanza tembeleo lako au mara baada ya kumaliza tembeleo lako hili.&lt;/span&gt;
 </t>
   </si>
   <si>
@@ -724,7 +726,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -768,6 +770,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
@@ -821,7 +826,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -833,13 +838,13 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" t="s">
         <v>13</v>
-      </c>
-      <c r="G1" t="s">
-        <v>14</v>
       </c>
       <c r="H1" t="s">
         <v>15</v>
@@ -857,10 +862,10 @@
         <v>19</v>
       </c>
       <c r="M1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="O1" t="s">
         <v>23</v>
@@ -892,7 +897,7 @@
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
         <v>28</v>
@@ -900,18 +905,18 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
         <v>41</v>
@@ -922,7 +927,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
@@ -936,7 +941,7 @@
         <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
@@ -952,7 +957,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>46</v>
@@ -966,18 +971,18 @@
         <v>47</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G10" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>1</v>
@@ -988,10 +993,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>28</v>
@@ -1016,36 +1021,36 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C15" s="1"/>
       <c r="F15" s="1"/>
       <c r="L15" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C16" s="1"/>
       <c r="F16" s="1"/>
       <c r="L16" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C17" s="1"/>
       <c r="F17" s="1"/>
@@ -1055,68 +1060,68 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C18" s="1"/>
       <c r="F18" s="1"/>
       <c r="L18" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>102</v>
@@ -1150,7 +1155,7 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>104</v>
@@ -1184,7 +1189,7 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B24" s="8" t="s">
         <v>106</v>
@@ -1218,7 +1223,7 @@
     </row>
     <row r="25">
       <c r="A25" s="8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>108</v>
@@ -1247,7 +1252,7 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>110</v>
@@ -1281,7 +1286,7 @@
     </row>
     <row r="27">
       <c r="A27" s="11" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>112</v>
@@ -1295,7 +1300,7 @@
     </row>
     <row r="28">
       <c r="A28" s="11" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>114</v>
@@ -1309,7 +1314,7 @@
     </row>
     <row r="29">
       <c r="A29" s="11" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>116</v>
@@ -1323,7 +1328,7 @@
     </row>
     <row r="30">
       <c r="A30" s="11" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>118</v>
@@ -1371,10 +1376,10 @@
       <c r="B32" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="D32" s="15" t="s">
+      <c r="D32" s="16" t="s">
         <v>127</v>
       </c>
       <c r="E32" s="15"/>
@@ -1432,7 +1437,7 @@
         <v>131</v>
       </c>
       <c r="E34" s="5"/>
-      <c r="F34" s="16"/>
+      <c r="F34" s="17"/>
       <c r="G34" s="4" t="s">
         <v>132</v>
       </c>
@@ -1463,10 +1468,10 @@
       <c r="B35" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C35" s="17" t="s">
+      <c r="C35" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="D35" s="18" t="s">
+      <c r="D35" s="19" t="s">
         <v>135</v>
       </c>
       <c r="E35" s="7"/>
@@ -1499,10 +1504,10 @@
       <c r="B36" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="C36" s="17" t="s">
+      <c r="C36" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="D36" s="18" t="s">
+      <c r="D36" s="19" t="s">
         <v>138</v>
       </c>
       <c r="E36" s="7"/>
@@ -1538,7 +1543,7 @@
       <c r="C37" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="D37" s="19" t="s">
+      <c r="D37" s="20" t="s">
         <v>141</v>
       </c>
       <c r="E37" s="5"/>
@@ -1620,7 +1625,7 @@
       <c r="C40" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="D40" s="17" t="s">
+      <c r="D40" s="18" t="s">
         <v>145</v>
       </c>
       <c r="E40" s="2"/>
@@ -1633,16 +1638,16 @@
         <v>146</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D41" s="17" t="s">
+      <c r="D41" s="18" t="s">
         <v>148</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>149</v>
@@ -1704,7 +1709,7 @@
         <v>157</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>158</v>
@@ -1721,7 +1726,7 @@
         <v>161</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>162</v>
@@ -1730,7 +1735,7 @@
         <v>163</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G45" s="1"/>
       <c r="I45" s="2"/>
@@ -1751,7 +1756,7 @@
         <v>167</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G46" s="1"/>
       <c r="I46" s="2"/>
@@ -1773,7 +1778,7 @@
         <v>171</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G47" s="1"/>
       <c r="I47" s="2"/>
@@ -1795,7 +1800,7 @@
         <v>174</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G48" s="1"/>
       <c r="I48" s="2"/>
@@ -1844,7 +1849,7 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>178</v>
@@ -1856,24 +1861,24 @@
         <v>180</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F51" s="2"/>
       <c r="G51" s="1"/>
-      <c r="I51" s="20" t="s">
+      <c r="I51" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="J51" s="21" t="s">
+      <c r="J51" s="22" t="s">
         <v>182</v>
       </c>
-      <c r="K51" s="21" t="s">
+      <c r="K51" s="22" t="s">
         <v>183</v>
       </c>
       <c r="L51" s="1"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>184</v>
@@ -1885,14 +1890,14 @@
         <v>186</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F52" s="2"/>
       <c r="G52" s="1"/>
-      <c r="I52" s="20" t="s">
+      <c r="I52" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="J52" s="21" t="s">
+      <c r="J52" s="22" t="s">
         <v>187</v>
       </c>
       <c r="K52" s="2" t="s">
@@ -1902,7 +1907,7 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>189</v>
@@ -1914,14 +1919,14 @@
         <v>191</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="1"/>
-      <c r="I53" s="20" t="s">
+      <c r="I53" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="J53" s="21" t="s">
+      <c r="J53" s="22" t="s">
         <v>192</v>
       </c>
       <c r="K53" s="2" t="s">
@@ -1931,7 +1936,7 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>194</v>
@@ -1943,14 +1948,14 @@
         <v>196</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="1"/>
-      <c r="I54" s="20" t="s">
+      <c r="I54" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="J54" s="21" t="s">
+      <c r="J54" s="22" t="s">
         <v>197</v>
       </c>
       <c r="K54" s="2" t="s">
@@ -1960,7 +1965,7 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>199</v>
@@ -1972,7 +1977,7 @@
         <v>201</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2" t="s">
@@ -1984,7 +1989,7 @@
       <c r="J55" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="K55" s="21" t="s">
+      <c r="K55" s="22" t="s">
         <v>205</v>
       </c>
       <c r="L55" s="1"/>
@@ -2035,7 +2040,7 @@
         <v>157</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I58" s="2" t="s">
         <v>158</v>
@@ -2094,13 +2099,13 @@
         <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -2108,105 +2113,105 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>73</v>
@@ -2217,86 +2222,86 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>76</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>76</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -2313,7 +2318,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s">
         <v>7</v>
@@ -2322,31 +2327,31 @@
         <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C2" s="3" t="str">
         <f>TEXT(NOW(), "yyyy-mm-dd_HH-MM")</f>
-        <v>2020-04-15_12-02</v>
+        <v>2020-05-13_11-59</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed the telephone issue
</commit_message>
<xml_diff>
--- a/forms/app/death_report.xlsx
+++ b/forms/app/death_report.xlsx
@@ -1,19 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\D-tree\config-dtree-newrepo\config-dtree\forms\app\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6325"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="survey" sheetId="1" r:id="rId3"/>
-    <sheet state="visible" name="choices" sheetId="2" r:id="rId4"/>
-    <sheet state="visible" name="settings" sheetId="3" r:id="rId5"/>
+    <sheet name="survey" sheetId="1" r:id="rId1"/>
+    <sheet name="choices" sheetId="2" r:id="rId2"/>
+    <sheet name="settings" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="210">
   <si>
     <t>type</t>
   </si>
@@ -509,9 +517,6 @@
     <t>numbers</t>
   </si>
   <si>
-    <t>regex(.,'^0[0-9]{9}$')</t>
-  </si>
-  <si>
     <t>Use the following format 0XXXXXXXXX</t>
   </si>
   <si>
@@ -669,38 +674,54 @@
   </si>
   <si>
     <t>data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tel </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="7">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="8">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Roboto"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF1D1C1D"/>
       <name val="Slack-Lato"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Sans"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -708,7 +729,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -724,116 +745,345 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
     <border>
+      <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyFont="1" applyNumberFormat="1"/>
+  <cellXfs count="26">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4472C4"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Z61"/>
+  <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="23.29"/>
-    <col customWidth="1" min="2" max="2" width="20.0"/>
-    <col customWidth="1" min="3" max="3" width="31.14"/>
-    <col customWidth="1" min="4" max="4" width="22.57"/>
-    <col customWidth="1" min="6" max="6" width="72.14"/>
+    <col min="1" max="1" width="23.26953125" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="31.1328125" customWidth="1"/>
+    <col min="4" max="4" width="22.54296875" customWidth="1"/>
+    <col min="6" max="6" width="72.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:17" ht="15.75" customHeight="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -886,7 +1136,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:17" ht="15.75" customHeight="1">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -901,7 +1151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:17" ht="15.75" customHeight="1">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -912,7 +1162,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:17" ht="15.75" customHeight="1">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -923,7 +1173,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:17" ht="15.75" customHeight="1">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -934,7 +1184,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:17" ht="15.75" customHeight="1">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -945,7 +1195,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:17" ht="15.75" customHeight="1">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -953,7 +1203,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:17" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -964,7 +1214,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:17" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>21</v>
       </c>
@@ -975,7 +1225,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:17" ht="15.75" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
@@ -989,7 +1239,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:17" ht="15.75" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
@@ -1000,7 +1250,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:17" ht="15.75" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
@@ -1011,7 +1261,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:17" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="s">
         <v>27</v>
       </c>
@@ -1020,7 +1270,7 @@
       </c>
       <c r="C13" s="1"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:17" ht="15.75" customHeight="1">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1028,7 +1278,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:17" ht="15.75" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>34</v>
       </c>
@@ -1041,7 +1291,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:17" ht="15.75" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>34</v>
       </c>
@@ -1054,7 +1304,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:26" ht="15.75" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
@@ -1067,7 +1317,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:26" ht="15.75" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>34</v>
       </c>
@@ -1080,7 +1330,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:26" ht="15.75" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>34</v>
       </c>
@@ -1096,7 +1346,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:26" ht="15.75" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>34</v>
       </c>
@@ -1112,7 +1362,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:26" ht="13">
       <c r="A21" s="1" t="s">
         <v>34</v>
       </c>
@@ -1128,7 +1378,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:26" ht="13">
       <c r="A22" s="3" t="s">
         <v>34</v>
       </c>
@@ -1162,7 +1412,7 @@
       <c r="Y22" s="4"/>
       <c r="Z22" s="4"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:26" ht="13">
       <c r="A23" s="3" t="s">
         <v>34</v>
       </c>
@@ -1196,7 +1446,7 @@
       <c r="Y23" s="4"/>
       <c r="Z23" s="4"/>
     </row>
-    <row r="24">
+    <row r="24" spans="1:26" ht="13">
       <c r="A24" s="3" t="s">
         <v>34</v>
       </c>
@@ -1230,7 +1480,7 @@
       <c r="Y24" s="4"/>
       <c r="Z24" s="4"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:26" ht="13">
       <c r="A25" s="7" t="s">
         <v>34</v>
       </c>
@@ -1246,9 +1496,14 @@
       <c r="I25" s="4"/>
       <c r="J25" s="4"/>
       <c r="K25" s="4"/>
-      <c r="L25" s="9" t="s">
+      <c r="L25" s="23" t="s">
         <v>57</v>
       </c>
+      <c r="M25" s="24"/>
+      <c r="N25" s="24"/>
+      <c r="O25" s="24"/>
+      <c r="P25" s="24"/>
+      <c r="Q25" s="24"/>
       <c r="R25" s="4"/>
       <c r="S25" s="4"/>
       <c r="T25" s="4"/>
@@ -1259,7 +1514,7 @@
       <c r="Y25" s="4"/>
       <c r="Z25" s="4"/>
     </row>
-    <row r="26">
+    <row r="26" spans="1:26" ht="13">
       <c r="A26" s="3" t="s">
         <v>34</v>
       </c>
@@ -1293,210 +1548,210 @@
       <c r="Y26" s="4"/>
       <c r="Z26" s="4"/>
     </row>
-    <row r="27">
-      <c r="A27" s="10" t="s">
+    <row r="27" spans="1:26" ht="13">
+      <c r="A27" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="9" t="s">
         <v>60</v>
       </c>
       <c r="C27" s="2"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
-      <c r="L27" s="11" t="s">
+      <c r="L27" s="10" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:26" ht="13">
+      <c r="A28" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="9" t="s">
         <v>62</v>
       </c>
       <c r="C28" s="2"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
-      <c r="L28" s="11" t="s">
+      <c r="L28" s="10" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="10" t="s">
+    <row r="29" spans="1:26" ht="13">
+      <c r="A29" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="9" t="s">
         <v>64</v>
       </c>
       <c r="C29" s="2"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
-      <c r="L29" s="11" t="s">
+      <c r="L29" s="10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="10" t="s">
+    <row r="30" spans="1:26" ht="13">
+      <c r="A30" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="9" t="s">
         <v>66</v>
       </c>
       <c r="C30" s="2"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
-      <c r="L30" s="11" t="s">
+      <c r="L30" s="10" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="10" t="s">
+    <row r="31" spans="1:26" ht="13">
+      <c r="A31" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C31" s="12"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="13"/>
-      <c r="J31" s="13"/>
-      <c r="K31" s="13"/>
-      <c r="L31" s="14"/>
-      <c r="M31" s="13"/>
-      <c r="N31" s="13"/>
-      <c r="O31" s="13"/>
-      <c r="P31" s="13"/>
-      <c r="Q31" s="13"/>
-      <c r="R31" s="13"/>
-      <c r="S31" s="13"/>
-      <c r="T31" s="13"/>
-      <c r="U31" s="13"/>
-      <c r="V31" s="13"/>
-      <c r="W31" s="13"/>
-      <c r="X31" s="13"/>
-      <c r="Y31" s="13"/>
-      <c r="Z31" s="13"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="s">
+      <c r="C31" s="11"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
+      <c r="L31" s="13"/>
+      <c r="M31" s="12"/>
+      <c r="N31" s="12"/>
+      <c r="O31" s="12"/>
+      <c r="P31" s="12"/>
+      <c r="Q31" s="12"/>
+      <c r="R31" s="12"/>
+      <c r="S31" s="12"/>
+      <c r="T31" s="12"/>
+      <c r="U31" s="12"/>
+      <c r="V31" s="12"/>
+      <c r="W31" s="12"/>
+      <c r="X31" s="12"/>
+      <c r="Y31" s="12"/>
+      <c r="Z31" s="12"/>
+    </row>
+    <row r="32" spans="1:26" ht="13">
+      <c r="A32" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C32" s="12"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="13"/>
-      <c r="J32" s="13"/>
-      <c r="K32" s="13"/>
-      <c r="L32" s="14"/>
-      <c r="M32" s="13"/>
-      <c r="N32" s="13"/>
-      <c r="O32" s="13"/>
-      <c r="P32" s="13"/>
-      <c r="Q32" s="13"/>
-      <c r="R32" s="13"/>
-      <c r="S32" s="13"/>
-      <c r="T32" s="13"/>
-      <c r="U32" s="13"/>
-      <c r="V32" s="13"/>
-      <c r="W32" s="13"/>
-      <c r="X32" s="13"/>
-      <c r="Y32" s="13"/>
-      <c r="Z32" s="13"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="12" t="s">
+      <c r="C32" s="11"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="12"/>
+      <c r="L32" s="13"/>
+      <c r="M32" s="12"/>
+      <c r="N32" s="12"/>
+      <c r="O32" s="12"/>
+      <c r="P32" s="12"/>
+      <c r="Q32" s="12"/>
+      <c r="R32" s="12"/>
+      <c r="S32" s="12"/>
+      <c r="T32" s="12"/>
+      <c r="U32" s="12"/>
+      <c r="V32" s="12"/>
+      <c r="W32" s="12"/>
+      <c r="X32" s="12"/>
+      <c r="Y32" s="12"/>
+      <c r="Z32" s="12"/>
+    </row>
+    <row r="33" spans="1:26" ht="13">
+      <c r="A33" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="B33" s="12" t="s">
+      <c r="B33" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="C33" s="12" t="s">
+      <c r="C33" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="D33" s="15" t="s">
+      <c r="D33" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="E33" s="13"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
-      <c r="J33" s="13"/>
-      <c r="K33" s="13"/>
-      <c r="L33" s="12"/>
-      <c r="M33" s="13"/>
-      <c r="N33" s="13"/>
-      <c r="O33" s="13"/>
-      <c r="P33" s="13"/>
-      <c r="Q33" s="13"/>
-      <c r="R33" s="13"/>
-      <c r="S33" s="13"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="12" t="s">
+      <c r="E33" s="12"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="12"/>
+      <c r="L33" s="11"/>
+      <c r="M33" s="12"/>
+      <c r="N33" s="12"/>
+      <c r="O33" s="12"/>
+      <c r="P33" s="12"/>
+      <c r="Q33" s="12"/>
+      <c r="R33" s="12"/>
+      <c r="S33" s="12"/>
+    </row>
+    <row r="34" spans="1:26" ht="13">
+      <c r="A34" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B34" s="12" t="s">
+      <c r="B34" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="C34" s="16" t="s">
+      <c r="C34" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D34" s="16" t="s">
+      <c r="D34" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="E34" s="13"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="13"/>
-      <c r="J34" s="13"/>
-      <c r="K34" s="13"/>
-      <c r="L34" s="12"/>
-      <c r="M34" s="13"/>
-      <c r="N34" s="13"/>
-      <c r="O34" s="13"/>
-      <c r="P34" s="13"/>
-      <c r="Q34" s="13"/>
-      <c r="R34" s="13"/>
-      <c r="S34" s="13"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="s">
+      <c r="E34" s="12"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
+      <c r="L34" s="11"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="12"/>
+      <c r="P34" s="12"/>
+      <c r="Q34" s="12"/>
+      <c r="R34" s="12"/>
+      <c r="S34" s="12"/>
+    </row>
+    <row r="35" spans="1:26" ht="13">
+      <c r="A35" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="B35" s="12" t="s">
+      <c r="B35" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="C35" s="12"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="12"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
-      <c r="J35" s="13"/>
-      <c r="K35" s="13"/>
-      <c r="L35" s="12"/>
-      <c r="M35" s="13"/>
-      <c r="N35" s="13"/>
-      <c r="O35" s="13"/>
-      <c r="P35" s="13"/>
-      <c r="Q35" s="13"/>
-      <c r="R35" s="13"/>
-      <c r="S35" s="13"/>
-    </row>
-    <row r="36">
+      <c r="C35" s="11"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="11"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
+      <c r="K35" s="12"/>
+      <c r="L35" s="11"/>
+      <c r="M35" s="12"/>
+      <c r="N35" s="12"/>
+      <c r="O35" s="12"/>
+      <c r="P35" s="12"/>
+      <c r="Q35" s="12"/>
+      <c r="R35" s="12"/>
+      <c r="S35" s="12"/>
+    </row>
+    <row r="36" spans="1:26" ht="13">
       <c r="A36" s="3" t="s">
         <v>17</v>
       </c>
@@ -1510,7 +1765,7 @@
         <v>81</v>
       </c>
       <c r="E36" s="4"/>
-      <c r="F36" s="17"/>
+      <c r="F36" s="16"/>
       <c r="G36" s="3" t="s">
         <v>82</v>
       </c>
@@ -1534,17 +1789,17 @@
       <c r="Y36" s="4"/>
       <c r="Z36" s="4"/>
     </row>
-    <row r="37">
+    <row r="37" spans="1:26" ht="13">
       <c r="A37" s="3" t="s">
         <v>74</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C37" s="18" t="s">
+      <c r="C37" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="D37" s="19" t="s">
+      <c r="D37" s="18" t="s">
         <v>85</v>
       </c>
       <c r="E37" s="6"/>
@@ -1570,17 +1825,17 @@
       <c r="Y37" s="4"/>
       <c r="Z37" s="4"/>
     </row>
-    <row r="38">
+    <row r="38" spans="1:26" ht="13">
       <c r="A38" s="3" t="s">
         <v>74</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C38" s="18" t="s">
+      <c r="C38" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="D38" s="19" t="s">
+      <c r="D38" s="18" t="s">
         <v>88</v>
       </c>
       <c r="E38" s="6"/>
@@ -1606,7 +1861,7 @@
       <c r="Y38" s="4"/>
       <c r="Z38" s="4"/>
     </row>
-    <row r="39">
+    <row r="39" spans="1:26" ht="13">
       <c r="A39" s="3" t="s">
         <v>74</v>
       </c>
@@ -1616,7 +1871,7 @@
       <c r="C39" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D39" s="20" t="s">
+      <c r="D39" s="19" t="s">
         <v>91</v>
       </c>
       <c r="E39" s="4"/>
@@ -1642,7 +1897,7 @@
       <c r="Y39" s="4"/>
       <c r="Z39" s="4"/>
     </row>
-    <row r="40">
+    <row r="40" spans="1:26" ht="13">
       <c r="A40" s="3" t="s">
         <v>27</v>
       </c>
@@ -1674,7 +1929,7 @@
       <c r="Y40" s="4"/>
       <c r="Z40" s="4"/>
     </row>
-    <row r="41">
+    <row r="41" spans="1:26" ht="13">
       <c r="A41" s="2" t="s">
         <v>17</v>
       </c>
@@ -1688,7 +1943,7 @@
       <c r="F41" s="1"/>
       <c r="L41" s="1"/>
     </row>
-    <row r="42">
+    <row r="42" spans="1:26" ht="13">
       <c r="A42" s="2" t="s">
         <v>74</v>
       </c>
@@ -1698,7 +1953,7 @@
       <c r="C42" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D42" s="18" t="s">
+      <c r="D42" s="17" t="s">
         <v>95</v>
       </c>
       <c r="E42" s="2"/>
@@ -1706,7 +1961,7 @@
       <c r="G42" s="1"/>
       <c r="L42" s="1"/>
     </row>
-    <row r="43">
+    <row r="43" spans="1:26" ht="13">
       <c r="A43" s="2" t="s">
         <v>96</v>
       </c>
@@ -1716,7 +1971,7 @@
       <c r="C43" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D43" s="18" t="s">
+      <c r="D43" s="17" t="s">
         <v>99</v>
       </c>
       <c r="E43" s="2" t="s">
@@ -1728,7 +1983,7 @@
       <c r="G43" s="1"/>
       <c r="L43" s="1"/>
     </row>
-    <row r="44">
+    <row r="44" spans="1:26" ht="13">
       <c r="A44" s="2" t="s">
         <v>27</v>
       </c>
@@ -1744,7 +1999,7 @@
       <c r="J44" s="2"/>
       <c r="L44" s="1"/>
     </row>
-    <row r="45">
+    <row r="45" spans="1:26" ht="13">
       <c r="A45" s="2" t="s">
         <v>17</v>
       </c>
@@ -1768,7 +2023,7 @@
       <c r="J45" s="2"/>
       <c r="L45" s="1"/>
     </row>
-    <row r="46">
+    <row r="46" spans="1:26" ht="13">
       <c r="A46" s="2" t="s">
         <v>106</v>
       </c>
@@ -1794,7 +2049,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:26" ht="13">
       <c r="A47" s="2" t="s">
         <v>113</v>
       </c>
@@ -1815,7 +2070,7 @@
       <c r="J47" s="2"/>
       <c r="L47" s="1"/>
     </row>
-    <row r="48">
+    <row r="48" spans="1:26" ht="13">
       <c r="A48" s="2" t="s">
         <v>117</v>
       </c>
@@ -1837,7 +2092,7 @@
       <c r="K48" s="2"/>
       <c r="L48" s="1"/>
     </row>
-    <row r="49">
+    <row r="49" spans="1:12" ht="13">
       <c r="A49" s="2" t="s">
         <v>121</v>
       </c>
@@ -1859,7 +2114,7 @@
       <c r="K49" s="2"/>
       <c r="L49" s="1"/>
     </row>
-    <row r="50">
+    <row r="50" spans="1:12" ht="13">
       <c r="A50" s="2" t="s">
         <v>121</v>
       </c>
@@ -1881,7 +2136,7 @@
       <c r="K50" s="2"/>
       <c r="L50" s="1"/>
     </row>
-    <row r="51">
+    <row r="51" spans="1:12" ht="13">
       <c r="A51" s="2" t="s">
         <v>27</v>
       </c>
@@ -1896,7 +2151,7 @@
       <c r="J51" s="2"/>
       <c r="L51" s="1"/>
     </row>
-    <row r="52">
+    <row r="52" spans="1:12" ht="13">
       <c r="A52" s="2" t="s">
         <v>17</v>
       </c>
@@ -1920,7 +2175,7 @@
       <c r="J52" s="2"/>
       <c r="L52" s="1"/>
     </row>
-    <row r="53">
+    <row r="53" spans="1:12" ht="13">
       <c r="A53" s="2" t="s">
         <v>21</v>
       </c>
@@ -1938,18 +2193,18 @@
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="1"/>
-      <c r="I53" s="21" t="s">
+      <c r="I53" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="J53" s="22" t="s">
+      <c r="J53" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="K53" s="22" t="s">
+      <c r="K53" s="21" t="s">
         <v>136</v>
       </c>
       <c r="L53" s="1"/>
     </row>
-    <row r="54">
+    <row r="54" spans="1:12" ht="13">
       <c r="A54" s="2" t="s">
         <v>21</v>
       </c>
@@ -1967,10 +2222,10 @@
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="1"/>
-      <c r="I54" s="21" t="s">
+      <c r="I54" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="J54" s="22" t="s">
+      <c r="J54" s="21" t="s">
         <v>140</v>
       </c>
       <c r="K54" s="2" t="s">
@@ -1978,7 +2233,7 @@
       </c>
       <c r="L54" s="1"/>
     </row>
-    <row r="55">
+    <row r="55" spans="1:12" ht="13">
       <c r="A55" s="2" t="s">
         <v>21</v>
       </c>
@@ -1996,10 +2251,10 @@
       </c>
       <c r="F55" s="2"/>
       <c r="G55" s="1"/>
-      <c r="I55" s="21" t="s">
+      <c r="I55" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="J55" s="22" t="s">
+      <c r="J55" s="21" t="s">
         <v>145</v>
       </c>
       <c r="K55" s="2" t="s">
@@ -2007,7 +2262,7 @@
       </c>
       <c r="L55" s="1"/>
     </row>
-    <row r="56">
+    <row r="56" spans="1:12" ht="13">
       <c r="A56" s="2" t="s">
         <v>21</v>
       </c>
@@ -2025,10 +2280,10 @@
       </c>
       <c r="F56" s="2"/>
       <c r="G56" s="1"/>
-      <c r="I56" s="21" t="s">
+      <c r="I56" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="J56" s="22" t="s">
+      <c r="J56" s="21" t="s">
         <v>150</v>
       </c>
       <c r="K56" s="2" t="s">
@@ -2036,9 +2291,9 @@
       </c>
       <c r="L56" s="1"/>
     </row>
-    <row r="57">
+    <row r="57" spans="1:12" ht="13">
       <c r="A57" s="2" t="s">
-        <v>21</v>
+        <v>209</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>152</v>
@@ -2056,18 +2311,18 @@
       <c r="G57" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="I57" s="2" t="s">
+      <c r="I57" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="J57" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="J57" s="10" t="s">
+      <c r="K57" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="K57" s="22" t="s">
-        <v>158</v>
-      </c>
       <c r="L57" s="1"/>
     </row>
-    <row r="58">
+    <row r="58" spans="1:12" ht="13">
       <c r="A58" s="2" t="s">
         <v>27</v>
       </c>
@@ -2082,29 +2337,29 @@
       <c r="J58" s="2"/>
       <c r="L58" s="1"/>
     </row>
-    <row r="59">
+    <row r="59" spans="1:12" ht="13">
       <c r="A59" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>19</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:12" ht="13">
       <c r="A60" s="2" t="s">
         <v>106</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>108</v>
@@ -2125,37 +2380,39 @@
         <v>112</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:12" ht="13">
       <c r="A61" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="L25:Q25"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="35.57"/>
-    <col customWidth="1" min="2" max="2" width="18.29"/>
-    <col customWidth="1" min="3" max="3" width="33.14"/>
+    <col min="1" max="1" width="35.54296875" customWidth="1"/>
+    <col min="2" max="2" width="18.26953125" customWidth="1"/>
+    <col min="3" max="3" width="33.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" ht="15.75" customHeight="1">
       <c r="A1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -2167,267 +2424,268 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>100</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D2" t="s">
         <v>164</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="3" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A3" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" t="s">
         <v>167</v>
       </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="4" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A4" s="2" t="s">
         <v>168</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>169</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>100</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D4" t="s">
         <v>164</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="5" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="s">
+      <c r="C5" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="D5" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="7">
+    </row>
+    <row r="7" spans="1:4" ht="15.75" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>97</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="8">
+    </row>
+    <row r="8" spans="1:4" ht="15.75" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>97</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="9">
+    </row>
+    <row r="9" spans="1:4" ht="15.75" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>97</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="10">
+    </row>
+    <row r="10" spans="1:4" ht="15.75" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>97</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="11">
+    </row>
+    <row r="11" spans="1:4" ht="15.75" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>97</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="12">
+    </row>
+    <row r="12" spans="1:4" ht="15.75" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>114</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="13">
+    </row>
+    <row r="13" spans="1:4" ht="15.75" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>114</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="14">
+    </row>
+    <row r="14" spans="1:4" ht="15.75" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>114</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="15">
+    </row>
+    <row r="15" spans="1:4" ht="15.75" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>114</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="16">
+    </row>
+    <row r="16" spans="1:4" ht="15.75" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>114</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1">
       <c r="A1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B1" t="s">
         <v>200</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>201</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>202</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>203</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>204</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="2" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A2" s="1" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="22" t="str">
+        <f ca="1">TEXT(NOW(), "yyyy-mm-dd_HH-MM")</f>
+        <v>2021-01-29 9-24</v>
+      </c>
+      <c r="D2" t="s">
         <v>207</v>
       </c>
-      <c r="C2" s="23" t="str">
-        <f>TEXT(NOW(), "yyyy-mm-dd_HH-MM")</f>
-        <v>2020-10-06_12-18</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>208</v>
       </c>
-      <c r="E2" t="s">
-        <v>209</v>
-      </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove enabel in maintenance (#107) (#105)
* Remove enabel in maintenance (#107)

* Worked on PR review changes (#108)
</commit_message>
<xml_diff>
--- a/forms/app/death_report.xlsx
+++ b/forms/app/death_report.xlsx
@@ -1,27 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20382"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\D-tree\config-dtree-newrepo\config-dtree\forms\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B0661E-5F75-4684-BC40-CDB393940144}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6325"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
     <sheet name="choices" sheetId="2" r:id="rId2"/>
     <sheet name="settings" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="244">
   <si>
     <t>type</t>
   </si>
@@ -514,9 +515,6 @@
     <t>Namba ya Simu</t>
   </si>
   <si>
-    <t>numbers</t>
-  </si>
-  <si>
     <t>Use the following format 0XXXXXXXXX</t>
   </si>
   <si>
@@ -526,9 +524,6 @@
     <t>other</t>
   </si>
   <si>
-    <t>not(${sex} = "female" and ${age_in_years} &gt;= 12 and ${reason_death} = "pregnancy_delivery")</t>
-  </si>
-  <si>
     <t>date_of_death_other</t>
   </si>
   <si>
@@ -676,14 +671,122 @@
     <t>data</t>
   </si>
   <si>
-    <t xml:space="preserve">tel </t>
+    <t>reason_death_child</t>
+  </si>
+  <si>
+    <t>What is the reason for the child's death?</t>
+  </si>
+  <si>
+    <t>select_one reason_death_child</t>
+  </si>
+  <si>
+    <t xml:space="preserve">respiratory_infection </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Respiratory Infection </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maradhi ya kupumua </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diarhoea </t>
+  </si>
+  <si>
+    <t xml:space="preserve">diarhoea </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kuharisha </t>
+  </si>
+  <si>
+    <t xml:space="preserve">malaria </t>
+  </si>
+  <si>
+    <t>Malaria</t>
+  </si>
+  <si>
+    <t>malnutrition</t>
+  </si>
+  <si>
+    <t>Malnutrition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utapia mlo </t>
+  </si>
+  <si>
+    <t xml:space="preserve">other </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other </t>
+  </si>
+  <si>
+    <t>select_one where_death_child</t>
+  </si>
+  <si>
+    <t>where_death_child</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Where did the child die? </t>
+  </si>
+  <si>
+    <t>Amefia wapi ?</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If other, please specify </t>
+  </si>
+  <si>
+    <t>Tafadhali taja sababu ya kifo</t>
+  </si>
+  <si>
+    <t>where_death_child_other</t>
+  </si>
+  <si>
+    <t>reason_death_child_other</t>
+  </si>
+  <si>
+    <t>where_death_woman_other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">selected(${where_death},"other") </t>
+  </si>
+  <si>
+    <t>Tafadhali taja</t>
+  </si>
+  <si>
+    <t>reason_death_other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">selected(${reason_death},"other")  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">${age_in_years} &lt; 12 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">${age_in_years} &lt; 12  and selected(${where_death_child},"other") </t>
+  </si>
+  <si>
+    <t xml:space="preserve">${age_in_years} &lt; 12  and selected(${reason_death_child},"other") </t>
+  </si>
+  <si>
+    <t>not(${reason_death} = "pregnancy_delivery")</t>
+  </si>
+  <si>
+    <t>regex(.,'^[0oO][0-9oO]{9}$')</t>
+  </si>
+  <si>
+    <t>next_of_kin_phone_raw</t>
+  </si>
+  <si>
+    <t>translate (translate (${next_of_kin_phone_raw}, "o","0"), "O","0")</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -692,10 +795,12 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -706,6 +811,7 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -716,12 +822,6 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Sans"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -760,10 +860,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -787,12 +888,17 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{56A7917D-47CA-4947-AA3A-2354174BC1E6}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1069,18 +1175,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z61"/>
+  <dimension ref="A1:Z68"/>
   <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="23.26953125" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="1" max="1" width="25.40625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.86328125" customWidth="1"/>
     <col min="3" max="3" width="31.1328125" customWidth="1"/>
     <col min="4" max="4" width="22.54296875" customWidth="1"/>
-    <col min="6" max="6" width="72.1328125" customWidth="1"/>
+    <col min="6" max="6" width="74.2265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" customHeight="1">
@@ -1496,14 +1602,14 @@
       <c r="I25" s="4"/>
       <c r="J25" s="4"/>
       <c r="K25" s="4"/>
-      <c r="L25" s="23" t="s">
+      <c r="L25" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="M25" s="24"/>
-      <c r="N25" s="24"/>
-      <c r="O25" s="24"/>
-      <c r="P25" s="24"/>
-      <c r="Q25" s="24"/>
+      <c r="M25" s="27"/>
+      <c r="N25" s="27"/>
+      <c r="O25" s="27"/>
+      <c r="P25" s="27"/>
+      <c r="Q25" s="27"/>
       <c r="R25" s="4"/>
       <c r="S25" s="4"/>
       <c r="T25" s="4"/>
@@ -1941,6 +2047,9 @@
       </c>
       <c r="D41" s="4"/>
       <c r="F41" s="1"/>
+      <c r="G41" t="s">
+        <v>82</v>
+      </c>
       <c r="L41" s="1"/>
     </row>
     <row r="42" spans="1:26" ht="13">
@@ -1971,7 +2080,7 @@
       <c r="C43" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D43" s="17" t="s">
+      <c r="D43" s="2" t="s">
         <v>99</v>
       </c>
       <c r="E43" s="2" t="s">
@@ -1983,105 +2092,107 @@
       <c r="G43" s="1"/>
       <c r="L43" s="1"/>
     </row>
-    <row r="44" spans="1:26" ht="13">
+    <row r="44" spans="1:26" s="24" customFormat="1" ht="13">
       <c r="A44" s="2" t="s">
-        <v>27</v>
+        <v>227</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
+        <v>235</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>236</v>
+      </c>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
-      <c r="L44" s="1"/>
+      <c r="K44" s="2"/>
     </row>
     <row r="45" spans="1:26" ht="13">
       <c r="A45" s="2" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>104</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
       <c r="E45" s="2"/>
-      <c r="F45" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>82</v>
-      </c>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
       <c r="L45" s="1"/>
     </row>
     <row r="46" spans="1:26" ht="13">
       <c r="A46" s="2" t="s">
-        <v>106</v>
+        <v>17</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="I46" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="J46" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>112</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+      <c r="L46" s="1"/>
     </row>
     <row r="47" spans="1:26" ht="13">
       <c r="A47" s="2" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G47" s="1"/>
-      <c r="I47" s="2"/>
-      <c r="J47" s="2"/>
-      <c r="L47" s="1"/>
+      <c r="I47" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="48" spans="1:26" ht="13">
       <c r="A48" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>100</v>
@@ -2089,43 +2200,43 @@
       <c r="G48" s="1"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
-      <c r="K48" s="2"/>
       <c r="L48" s="1"/>
     </row>
-    <row r="49" spans="1:12" ht="13">
+    <row r="49" spans="1:26" s="24" customFormat="1" ht="13">
       <c r="A49" s="2" t="s">
-        <v>121</v>
+        <v>227</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>122</v>
+        <v>232</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>123</v>
+        <v>228</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>124</v>
+        <v>234</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G49" s="1"/>
+      <c r="F49" s="2" t="s">
+        <v>233</v>
+      </c>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
-      <c r="L49" s="1"/>
-    </row>
-    <row r="50" spans="1:12" ht="13">
+    </row>
+    <row r="50" spans="1:26" ht="13">
       <c r="A50" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>100</v>
@@ -2136,115 +2247,101 @@
       <c r="K50" s="2"/>
       <c r="L50" s="1"/>
     </row>
-    <row r="51" spans="1:12" ht="13">
+    <row r="51" spans="1:26" ht="13">
       <c r="A51" s="2" t="s">
-        <v>27</v>
+        <v>121</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="G51" s="2"/>
+        <v>122</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="G51" s="1"/>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
+      <c r="K51" s="2"/>
       <c r="L51" s="1"/>
     </row>
-    <row r="52" spans="1:12" ht="13">
+    <row r="52" spans="1:26" ht="13">
       <c r="A52" s="2" t="s">
-        <v>17</v>
+        <v>121</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>82</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="G52" s="1"/>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
       <c r="L52" s="1"/>
     </row>
-    <row r="53" spans="1:12" ht="13">
+    <row r="53" spans="1:26" ht="13">
       <c r="A53" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="F53" s="2"/>
-      <c r="G53" s="1"/>
-      <c r="I53" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="J53" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="K53" s="21" t="s">
-        <v>136</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="2"/>
       <c r="L53" s="1"/>
     </row>
-    <row r="54" spans="1:12" ht="13">
+    <row r="54" spans="1:26" ht="13">
       <c r="A54" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="F54" s="2"/>
-      <c r="G54" s="1"/>
-      <c r="I54" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="J54" s="21" t="s">
-        <v>140</v>
-      </c>
-      <c r="K54" s="2" t="s">
-        <v>141</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="I54" s="2"/>
+      <c r="J54" s="2"/>
       <c r="L54" s="1"/>
     </row>
-    <row r="55" spans="1:12" ht="13">
+    <row r="55" spans="1:26" ht="13">
       <c r="A55" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>100</v>
@@ -2255,25 +2352,25 @@
         <v>134</v>
       </c>
       <c r="J55" s="21" t="s">
-        <v>145</v>
-      </c>
-      <c r="K55" s="2" t="s">
-        <v>146</v>
+        <v>135</v>
+      </c>
+      <c r="K55" s="21" t="s">
+        <v>136</v>
       </c>
       <c r="L55" s="1"/>
     </row>
-    <row r="56" spans="1:12" ht="13">
+    <row r="56" spans="1:26" ht="13">
       <c r="A56" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>100</v>
@@ -2284,108 +2381,290 @@
         <v>134</v>
       </c>
       <c r="J56" s="21" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="L56" s="1"/>
     </row>
-    <row r="57" spans="1:12" ht="13">
+    <row r="57" spans="1:26" ht="13">
       <c r="A57" s="2" t="s">
-        <v>209</v>
+        <v>21</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>100</v>
       </c>
       <c r="F57" s="2"/>
-      <c r="G57" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="I57" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="J57" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="K57" s="21" t="s">
-        <v>157</v>
+      <c r="G57" s="1"/>
+      <c r="I57" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="J57" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>146</v>
       </c>
       <c r="L57" s="1"/>
     </row>
-    <row r="58" spans="1:12" ht="13">
+    <row r="58" spans="1:26" ht="13">
       <c r="A58" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="C58" s="2"/>
-      <c r="E58" s="2"/>
+        <v>147</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>100</v>
+      </c>
       <c r="F58" s="2"/>
       <c r="G58" s="1"/>
-      <c r="I58" s="2"/>
-      <c r="J58" s="2"/>
+      <c r="I58" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="J58" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>151</v>
+      </c>
       <c r="L58" s="1"/>
     </row>
-    <row r="59" spans="1:12" ht="13">
+    <row r="59" spans="1:26" ht="13">
       <c r="A59" s="2" t="s">
-        <v>17</v>
+        <v>227</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>158</v>
+        <v>242</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="G59" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" ht="13">
-      <c r="A60" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E60" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E59" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="I60" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="J60" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="K60" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" ht="13">
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="I59" s="28" t="s">
+        <v>241</v>
+      </c>
+      <c r="J59" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="K59" s="21" t="s">
+        <v>156</v>
+      </c>
+      <c r="L59" s="1"/>
+    </row>
+    <row r="60" spans="1:26" s="25" customFormat="1" ht="13.5" customHeight="1">
+      <c r="A60" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B60" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="C60" s="21"/>
+      <c r="D60" s="21"/>
+      <c r="E60" s="29"/>
+      <c r="F60" s="29"/>
+      <c r="G60" s="29"/>
+      <c r="H60" s="29"/>
+      <c r="I60" s="28"/>
+      <c r="J60" s="21"/>
+      <c r="K60" s="21"/>
+      <c r="L60" s="29" t="s">
+        <v>243</v>
+      </c>
+      <c r="M60" s="29"/>
+      <c r="N60" s="29"/>
+      <c r="O60" s="29"/>
+      <c r="P60" s="29"/>
+      <c r="Q60" s="29"/>
+      <c r="R60" s="29"/>
+      <c r="S60" s="29"/>
+      <c r="T60" s="29"/>
+      <c r="U60" s="29"/>
+      <c r="V60" s="29"/>
+      <c r="W60" s="29"/>
+      <c r="X60" s="29"/>
+      <c r="Y60" s="29"/>
+      <c r="Z60" s="29"/>
+    </row>
+    <row r="61" spans="1:26" ht="13">
       <c r="A61" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B61" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="1"/>
+      <c r="I61" s="2"/>
+      <c r="J61" s="2"/>
+      <c r="L61" s="1"/>
+    </row>
+    <row r="62" spans="1:26" ht="13">
+      <c r="A62" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="63" spans="1:26" ht="13">
+      <c r="A63" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B63" s="2" t="s">
         <v>158</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="64" spans="1:26" s="23" customFormat="1" ht="13">
+      <c r="A64" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I64" s="2"/>
+      <c r="J64" s="2"/>
+      <c r="K64" s="2"/>
+    </row>
+    <row r="65" spans="1:11" s="24" customFormat="1" ht="13">
+      <c r="A65" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="I65" s="2"/>
+      <c r="J65" s="2"/>
+      <c r="K65" s="2"/>
+    </row>
+    <row r="66" spans="1:11" s="23" customFormat="1" ht="13">
+      <c r="A66" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="D66" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I66" s="2"/>
+      <c r="J66" s="2"/>
+      <c r="K66" s="2"/>
+    </row>
+    <row r="67" spans="1:11" s="23" customFormat="1" ht="13">
+      <c r="A67" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="I67" s="2"/>
+      <c r="J67" s="2"/>
+      <c r="K67" s="2"/>
+    </row>
+    <row r="68" spans="1:11" ht="13">
+      <c r="A68" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -2398,11 +2677,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="35.54296875" customWidth="1"/>
@@ -2412,7 +2691,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1">
       <c r="A1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -2426,72 +2705,72 @@
     </row>
     <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>100</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D3" t="s">
         <v>165</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="D3" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>100</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D5" t="s">
         <v>165</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="D5" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" customHeight="1">
@@ -2499,13 +2778,13 @@
         <v>97</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" customHeight="1">
@@ -2513,13 +2792,13 @@
         <v>97</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" customHeight="1">
@@ -2527,13 +2806,13 @@
         <v>97</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75" customHeight="1">
@@ -2541,13 +2820,13 @@
         <v>97</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>181</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1">
@@ -2555,13 +2834,13 @@
         <v>97</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.75" customHeight="1">
@@ -2569,13 +2848,13 @@
         <v>114</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>186</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" customHeight="1">
@@ -2583,13 +2862,13 @@
         <v>114</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.75" customHeight="1">
@@ -2597,13 +2876,13 @@
         <v>114</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.75" customHeight="1">
@@ -2611,13 +2890,13 @@
         <v>114</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15.75" customHeight="1">
@@ -2625,13 +2904,139 @@
         <v>114</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" s="23" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>198</v>
+      <c r="C22" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" s="23" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" s="23" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" s="23" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -2640,7 +3045,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -2649,40 +3054,40 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" customHeight="1">
       <c r="A1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C1" t="s">
         <v>199</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>200</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>201</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>202</v>
-      </c>
-      <c r="E1" t="s">
-        <v>203</v>
-      </c>
-      <c r="F1" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C2" s="22" t="str">
         <f ca="1">TEXT(NOW(), "yyyy-mm-dd_HH-MM")</f>
-        <v>2021-01-29 9-24</v>
+        <v>2022-02-11 11-02</v>
       </c>
       <c r="D2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>